<commit_message>
Add fresh guard-only replicate and compact OOD Sankey
</commit_message>
<xml_diff>
--- a/figures/Figures_2_3_Source_Data.xlsx
+++ b/figures/Figures_2_3_Source_Data.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -27,12 +27,6 @@
       <name val="Arial"/>
       <color rgb="FF222222"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="FF222222"/>
-      <sz val="15"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -50,7 +44,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFD9D9D9"/>
+        <fgColor rgb="FFE6E6E6"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,16 +60,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -84,32 +80,29 @@
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -200,12 +193,12 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr sz="1350">
+              <a:rPr sz="1200" b="1">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>(a) Service-token ledger</a:t>
+              <a:t>(a) Reference agreement</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -216,7 +209,7 @@
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1350">
+            <a:defRPr sz="1200" b="1">
               <a:latin typeface="Arial"/>
               <a:ea typeface="Arial"/>
               <a:cs typeface="Arial"/>
@@ -231,17 +224,17 @@
     <plotArea>
       <barChart>
         <barDir val="col"/>
-        <grouping val="stacked"/>
+        <grouping val="clustered"/>
         <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>JEV tokens (millions)</v>
+            <v>Point estimate</v>
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="FFFFFF"/>
+              <a:srgbClr val="5A5A5A"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
               <a:solidFill>
@@ -252,7 +245,7 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'Data 2'!$B$26:$B$27</f>
+              <f>'Data 2'!$B$2:$B$4</f>
               <strCache>
                 <ptCount val="0"/>
               </strCache>
@@ -260,9 +253,9 @@
           </cat>
           <val>
             <numRef>
-              <f>'Data 2'!$C$26:$C$27</f>
+              <f>'Data 2'!$C$2:$C$4</f>
               <numCache>
-                <formatCode>0.00</formatCode>
+                <formatCode>0.00%</formatCode>
                 <ptCount val="0"/>
               </numCache>
             </numRef>
@@ -272,12 +265,17 @@
           <idx val="1"/>
           <order val="1"/>
           <tx>
-            <v>L2 tokens (millions)</v>
+            <v>95% lower</v>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="D9D9D9"/>
-            </a:solidFill>
+            <a:pattFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="upDiag">
+              <a:fgClr>
+                <a:srgbClr val="5A5A5A"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:srgbClr val="FFFFFF"/>
+              </a:bgClr>
+            </a:pattFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
               <a:solidFill>
                 <a:srgbClr val="222222"/>
@@ -287,7 +285,7 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'Data 2'!$B$26:$B$27</f>
+              <f>'Data 2'!$B$2:$B$4</f>
               <strCache>
                 <ptCount val="0"/>
               </strCache>
@@ -295,16 +293,15 @@
           </cat>
           <val>
             <numRef>
-              <f>'Data 2'!$D$26:$D$27</f>
+              <f>'Data 2'!$D$2:$D$4</f>
               <numCache>
-                <formatCode>0.00</formatCode>
+                <formatCode>0.00%</formatCode>
                 <ptCount val="0"/>
               </numCache>
             </numRef>
           </val>
         </ser>
-        <gapWidth val="85"/>
-        <overlap val="100"/>
+        <gapWidth val="110"/>
         <axId val="48650112"/>
         <axId val="48672768"/>
       </barChart>
@@ -332,7 +329,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1125">
+              <a:defRPr sz="975">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
@@ -350,22 +347,55 @@
         <axId val="48672768"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="3"/>
+          <max val="1.02"/>
           <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4763">
-              <a:solidFill>
-                <a:srgbClr val="D9D9D9"/>
-              </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
         </majorGridlines>
-        <numFmt formatCode="0.0" sourceLinked="0"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:r>
+                  <a:rPr sz="900">
+                    <a:latin typeface="Arial"/>
+                    <a:ea typeface="Arial"/>
+                    <a:cs typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>Agreement (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+            <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="900">
+                  <a:latin typeface="Arial"/>
+                  <a:ea typeface="Arial"/>
+                  <a:cs typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t>None</a:t>
+              </a:r>
+            </a:p>
+          </txPr>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <txPr>
@@ -373,7 +403,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1050">
+              <a:defRPr sz="900">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
@@ -396,7 +426,7 @@
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="975">
+            <a:defRPr sz="900">
               <a:latin typeface="Arial"/>
               <a:ea typeface="Arial"/>
               <a:cs typeface="Arial"/>
@@ -432,12 +462,12 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr sz="1350">
+              <a:rPr sz="1200" b="1">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>(b) Agreement and 95% interval</a:t>
+              <a:t>(b) Service-token use</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -448,7 +478,7 @@
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1350">
+            <a:defRPr sz="1200" b="1">
               <a:latin typeface="Arial"/>
               <a:ea typeface="Arial"/>
               <a:cs typeface="Arial"/>
@@ -463,17 +493,57 @@
     <plotArea>
       <barChart>
         <barDir val="col"/>
-        <grouping val="clustered"/>
+        <grouping val="stacked"/>
         <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>Estimate</v>
+            <v>JEV</v>
+          </tx>
+          <spPr>
+            <a:pattFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="upDiag">
+              <a:fgClr>
+                <a:srgbClr val="5A5A5A"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:srgbClr val="FFFFFF"/>
+              </a:bgClr>
+            </a:pattFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="222222"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <strRef>
+              <f>'Data 2'!$G$2:$G$3</f>
+              <strCache>
+                <ptCount val="0"/>
+              </strCache>
+            </strRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Data 2'!$H$2:$H$3</f>
+              <numCache>
+                <formatCode>0.00</formatCode>
+                <ptCount val="0"/>
+              </numCache>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>L2</v>
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="222222"/>
+              <a:srgbClr val="5A5A5A"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
               <a:solidFill>
@@ -484,7 +554,7 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'Data 2'!$G$26:$G$28</f>
+              <f>'Data 2'!$G$2:$G$3</f>
               <strCache>
                 <ptCount val="0"/>
               </strCache>
@@ -492,85 +562,16 @@
           </cat>
           <val>
             <numRef>
-              <f>'Data 2'!$H$26:$H$28</f>
+              <f>'Data 2'!$I$2:$I$3</f>
               <numCache>
-                <formatCode>0.00%</formatCode>
+                <formatCode>0.00</formatCode>
                 <ptCount val="0"/>
               </numCache>
             </numRef>
           </val>
         </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <v>95% lower</v>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="D9D9D9"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="222222"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'Data 2'!$G$26:$G$28</f>
-              <strCache>
-                <ptCount val="0"/>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data 2'!$I$26:$I$28</f>
-              <numCache>
-                <formatCode>0.00%</formatCode>
-                <ptCount val="0"/>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <v>95% upper</v>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="FFFFFF"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="222222"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'Data 2'!$G$26:$G$28</f>
-              <strCache>
-                <ptCount val="0"/>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data 2'!$J$26:$J$28</f>
-              <numCache>
-                <formatCode>0.00%</formatCode>
-                <ptCount val="0"/>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="85"/>
+        <gapWidth val="135"/>
+        <overlap val="100"/>
         <axId val="48650112"/>
         <axId val="48672768"/>
       </barChart>
@@ -598,7 +599,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1125">
+              <a:defRPr sz="975">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
@@ -616,22 +617,55 @@
         <axId val="48672768"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="1.02"/>
-          <min val="0.88"/>
+          <max val="3.05"/>
+          <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4763">
-              <a:solidFill>
-                <a:srgbClr val="D9D9D9"/>
-              </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
         </majorGridlines>
-        <numFmt formatCode="0%" sourceLinked="0"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:r>
+                  <a:rPr sz="900">
+                    <a:latin typeface="Arial"/>
+                    <a:ea typeface="Arial"/>
+                    <a:cs typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>Tokens (millions)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+            <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="900">
+                  <a:latin typeface="Arial"/>
+                  <a:ea typeface="Arial"/>
+                  <a:cs typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t>None</a:t>
+              </a:r>
+            </a:p>
+          </txPr>
+        </title>
+        <numFmt formatCode="0.0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <txPr>
@@ -639,7 +673,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1050">
+              <a:defRPr sz="900">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
@@ -662,7 +696,7 @@
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="975">
+            <a:defRPr sz="900">
               <a:latin typeface="Arial"/>
               <a:ea typeface="Arial"/>
               <a:cs typeface="Arial"/>
@@ -698,12 +732,12 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr sz="1350">
+              <a:rPr sz="1200" b="1">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>(a) Reference agreement</a:t>
+              <a:t>(a) Selective invocation by cohort</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -714,7 +748,7 @@
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1350">
+            <a:defRPr sz="1200" b="1">
               <a:latin typeface="Arial"/>
               <a:ea typeface="Arial"/>
               <a:cs typeface="Arial"/>
@@ -735,11 +769,51 @@
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>Agreement</v>
+            <v>JEV</v>
+          </tx>
+          <spPr>
+            <a:pattFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="upDiag">
+              <a:fgClr>
+                <a:srgbClr val="5A5A5A"/>
+              </a:fgClr>
+              <a:bgClr>
+                <a:srgbClr val="FFFFFF"/>
+              </a:bgClr>
+            </a:pattFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="222222"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <strRef>
+              <f>'Data 3'!$B$2:$B$4</f>
+              <strCache>
+                <ptCount val="0"/>
+              </strCache>
+            </strRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Data 3'!$F$2:$F$4</f>
+              <numCache>
+                <formatCode>0.00%</formatCode>
+                <ptCount val="0"/>
+              </numCache>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>L2</v>
           </tx>
           <spPr>
             <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="222222"/>
+              <a:srgbClr val="5A5A5A"/>
             </a:solidFill>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
               <a:solidFill>
@@ -750,7 +824,7 @@
           </spPr>
           <cat>
             <strRef>
-              <f>'Data 3'!$B$26:$B$28</f>
+              <f>'Data 3'!$B$2:$B$4</f>
               <strCache>
                 <ptCount val="0"/>
               </strCache>
@@ -758,7 +832,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'Data 3'!$D$26:$D$28</f>
+              <f>'Data 3'!$G$2:$G$4</f>
               <numCache>
                 <formatCode>0.00%</formatCode>
                 <ptCount val="0"/>
@@ -766,7 +840,7 @@
             </numRef>
           </val>
         </ser>
-        <gapWidth val="85"/>
+        <gapWidth val="110"/>
         <axId val="48650112"/>
         <axId val="48672768"/>
       </barChart>
@@ -794,7 +868,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1125">
+              <a:defRPr sz="975">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
@@ -812,21 +886,54 @@
         <axId val="48672768"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="1.1"/>
+          <max val="1.05"/>
           <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4763">
-              <a:solidFill>
-                <a:srgbClr val="D9D9D9"/>
-              </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
         </majorGridlines>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:r>
+                  <a:rPr sz="900">
+                    <a:latin typeface="Arial"/>
+                    <a:ea typeface="Arial"/>
+                    <a:cs typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>Invocation rate (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+            <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="900">
+                  <a:latin typeface="Arial"/>
+                  <a:ea typeface="Arial"/>
+                  <a:cs typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t>None</a:t>
+              </a:r>
+            </a:p>
+          </txPr>
+        </title>
         <numFmt formatCode="0%" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -835,7 +942,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1050">
+              <a:defRPr sz="900">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
@@ -850,6 +957,26 @@
         <crossBetween val="between"/>
       </valAx>
     </plotArea>
+    <legend>
+      <legendPos val="b"/>
+      <overlay val="0"/>
+      <txPr>
+        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:pPr>
+            <a:defRPr sz="900">
+              <a:latin typeface="Arial"/>
+              <a:ea typeface="Arial"/>
+              <a:cs typeface="Arial"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:r>
+            <a:t>None</a:t>
+          </a:r>
+        </a:p>
+      </txPr>
+    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
@@ -874,12 +1001,12 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
-              <a:rPr sz="1350">
+              <a:rPr sz="1200" b="1">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
               </a:rPr>
-              <a:t>(b) Token saving</a:t>
+              <a:t>(b) Resource-quality operating regimes</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -890,7 +1017,7 @@
         <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
         <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:pPr>
-            <a:defRPr sz="1350">
+            <a:defRPr sz="1200" b="1">
               <a:latin typeface="Arial"/>
               <a:ea typeface="Arial"/>
               <a:cs typeface="Arial"/>
@@ -903,53 +1030,240 @@
       </txPr>
     </title>
     <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
+      <scatterChart>
+        <scatterStyle val="marker"/>
         <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <v>Token saving</v>
+            <v>Natural</v>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="222222"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="11430">
               <a:solidFill>
                 <a:srgbClr val="222222"/>
               </a:solidFill>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <cat>
-            <strRef>
-              <f>'Data 3'!$B$26:$B$28</f>
-              <strCache>
-                <ptCount val="0"/>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
+          <marker>
+            <symbol val="circle"/>
+            <size val="11"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="222222"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <txPr>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr sz="825">
+                    <a:solidFill>
+                      <a:srgbClr val="222222"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                    <a:ea typeface="Arial"/>
+                    <a:cs typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t>None</a:t>
+                </a:r>
+              </a:p>
+            </txPr>
+            <dLblPos val="l"/>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="1"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+            <showLeaderLines val="0"/>
+          </dLbls>
+          <xVal>
             <numRef>
-              <f>'Data 3'!$H$26:$H$28</f>
+              <f>'Data 3'!$M$2:$M$4</f>
               <numCache>
                 <formatCode>0.00%</formatCode>
                 <ptCount val="0"/>
               </numCache>
             </numRef>
-          </val>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Data 3'!$N$2:$N$4</f>
+              <numCache>
+                <formatCode>0.00%</formatCode>
+                <ptCount val="0"/>
+              </numCache>
+            </numRef>
+          </yVal>
         </ser>
-        <gapWidth val="85"/>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Stress</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="11430">
+              <a:solidFill>
+                <a:srgbClr val="222222"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="diamond"/>
+            <size val="11"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="222222"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <txPr>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr sz="825">
+                    <a:solidFill>
+                      <a:srgbClr val="222222"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                    <a:ea typeface="Arial"/>
+                    <a:cs typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t>None</a:t>
+                </a:r>
+              </a:p>
+            </txPr>
+            <dLblPos val="r"/>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="1"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+            <showLeaderLines val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'Data 3'!$M$2:$M$4</f>
+              <numCache>
+                <formatCode>0.00%</formatCode>
+                <ptCount val="0"/>
+              </numCache>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Data 3'!$O$2:$O$4</f>
+              <numCache>
+                <formatCode>0.00%</formatCode>
+                <ptCount val="0"/>
+              </numCache>
+            </numRef>
+          </yVal>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Policy OOD</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="11430">
+              <a:solidFill>
+                <a:srgbClr val="222222"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="square"/>
+            <size val="11"/>
+            <spPr>
+              <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:srgbClr val="5A5A5A"/>
+              </a:solidFill>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <dLbls>
+            <txPr>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr sz="825">
+                    <a:solidFill>
+                      <a:srgbClr val="222222"/>
+                    </a:solidFill>
+                    <a:latin typeface="Arial"/>
+                    <a:ea typeface="Arial"/>
+                    <a:cs typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:t>None</a:t>
+                </a:r>
+              </a:p>
+            </txPr>
+            <dLblPos val="t"/>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="0"/>
+            <showSerName val="1"/>
+            <showPercent val="0"/>
+            <showBubbleSize val="0"/>
+            <showLeaderLines val="0"/>
+          </dLbls>
+          <xVal>
+            <numRef>
+              <f>'Data 3'!$M$2:$M$4</f>
+              <numCache>
+                <formatCode>0.00%</formatCode>
+                <ptCount val="0"/>
+              </numCache>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'Data 3'!$P$2:$P$4</f>
+              <numCache>
+                <formatCode>0.00%</formatCode>
+                <ptCount val="0"/>
+              </numCache>
+            </numRef>
+          </yVal>
+        </ser>
         <axId val="48650112"/>
         <axId val="48672768"/>
-      </barChart>
-      <catAx>
+      </scatterChart>
+      <valAx>
         <axId val="48650112"/>
         <scaling>
           <orientation val="minMax"/>
+          <max val="1.05"/>
+          <min val="0"/>
         </scaling>
         <delete val="0"/>
         <axPos val="b"/>
@@ -961,7 +1275,42 @@
             </a:ln>
           </spPr>
         </majorGridlines>
-        <numFmt formatCode="General" sourceLinked="0"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:r>
+                  <a:rPr sz="900">
+                    <a:latin typeface="Arial"/>
+                    <a:ea typeface="Arial"/>
+                    <a:cs typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>Token use vs. full L2 (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+            <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="900">
+                  <a:latin typeface="Arial"/>
+                  <a:ea typeface="Arial"/>
+                  <a:cs typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t>None</a:t>
+              </a:r>
+            </a:p>
+          </txPr>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <tickLblPos val="nextTo"/>
@@ -970,7 +1319,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1125">
+              <a:defRPr sz="900">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
@@ -982,27 +1331,59 @@
           </a:p>
         </txPr>
         <crossAx val="48672768"/>
-        <lblOffset val="100"/>
-      </catAx>
+      </valAx>
       <valAx>
         <axId val="48672768"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="1"/>
-          <min val="-0.05"/>
+          <max val="1.02"/>
+          <min val="0.85"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4763">
-              <a:solidFill>
-                <a:srgbClr val="D9D9D9"/>
-              </a:solidFill>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
+              <a:noFill/>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
         </majorGridlines>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:r>
+                  <a:rPr sz="900">
+                    <a:latin typeface="Arial"/>
+                    <a:ea typeface="Arial"/>
+                    <a:cs typeface="Arial"/>
+                  </a:rPr>
+                  <a:t>Reference agreement (%)</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+          <overlay val="0"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
+            <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="900">
+                  <a:latin typeface="Arial"/>
+                  <a:ea typeface="Arial"/>
+                  <a:cs typeface="Arial"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t>None</a:t>
+              </a:r>
+            </a:p>
+          </txPr>
+        </title>
         <numFmt formatCode="0%" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -1011,7 +1392,7 @@
           <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
           <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
-              <a:defRPr sz="1050">
+              <a:defRPr sz="900">
                 <a:latin typeface="Arial"/>
                 <a:ea typeface="Arial"/>
                 <a:cs typeface="Arial"/>
@@ -1023,183 +1404,6 @@
           </a:p>
         </txPr>
         <crossAx val="48650112"/>
-        <crossBetween val="between"/>
-      </valAx>
-    </plotArea>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-  <spPr>
-    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-      <a:solidFill>
-        <a:srgbClr val="D9D9D9"/>
-      </a:solidFill>
-      <a:prstDash val="solid"/>
-    </a:ln>
-  </spPr>
-</chartSpace>
-</file>
-
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:r>
-              <a:rPr sz="1350">
-                <a:latin typeface="Arial"/>
-                <a:ea typeface="Arial"/>
-                <a:cs typeface="Arial"/>
-              </a:rPr>
-              <a:t>(c) L2 invocation</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-      <overlay val="0"/>
-      <txPr>
-        <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
-        <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-        <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:pPr>
-            <a:defRPr sz="1350">
-              <a:latin typeface="Arial"/>
-              <a:ea typeface="Arial"/>
-              <a:cs typeface="Arial"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:r>
-            <a:t>None</a:t>
-          </a:r>
-        </a:p>
-      </txPr>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <varyColors val="0"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <v>L2 rate</v>
-          </tx>
-          <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:srgbClr val="222222"/>
-            </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="222222"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <strRef>
-              <f>'Data 3'!$B$26:$B$28</f>
-              <strCache>
-                <ptCount val="0"/>
-              </strCache>
-            </strRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'Data 3'!$I$26:$I$28</f>
-              <numCache>
-                <formatCode>0.00%</formatCode>
-                <ptCount val="0"/>
-              </numCache>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="85"/>
-        <axId val="48650112"/>
-        <axId val="48672768"/>
-      </barChart>
-      <catAx>
-        <axId val="48650112"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="b"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="0">
-              <a:noFill/>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
-        <numFmt formatCode="General" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <tickLblPos val="nextTo"/>
-        <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="1125">
-                <a:latin typeface="Arial"/>
-                <a:ea typeface="Arial"/>
-                <a:cs typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-          </a:p>
-        </txPr>
-        <crossAx val="48672768"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="48672768"/>
-        <scaling>
-          <orientation val="minMax"/>
-          <max val="1.1"/>
-          <min val="0"/>
-        </scaling>
-        <delete val="0"/>
-        <axPos val="l"/>
-        <majorGridlines>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="4763">
-              <a:solidFill>
-                <a:srgbClr val="D9D9D9"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-        </majorGridlines>
-        <numFmt formatCode="0%" sourceLinked="0"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <txPr>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" anchorCtr="1"/>
-          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr sz="1050">
-                <a:latin typeface="Arial"/>
-                <a:ea typeface="Arial"/>
-                <a:cs typeface="Arial"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:t>None</a:t>
-            </a:r>
-          </a:p>
-        </txPr>
-        <crossAx val="48650112"/>
-        <crossBetween val="between"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -1285,7 +1489,7 @@
       <rowOff>0</rowOff>
     </from>
     <to>
-      <col>8</col>
+      <col>11</col>
       <colOff>0</colOff>
       <row>23</row>
       <rowOff>0</rowOff>
@@ -1306,13 +1510,13 @@
   </twoCellAnchor>
   <twoCellAnchor>
     <from>
-      <col>8</col>
+      <col>11</col>
       <colOff>0</colOff>
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
     <to>
-      <col>15</col>
+      <col>22</col>
       <colOff>0</colOff>
       <row>23</row>
       <rowOff>0</rowOff>
@@ -1326,33 +1530,6 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor>
-    <from>
-      <col>15</col>
-      <colOff>0</colOff>
-      <row>3</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>22</col>
-      <colOff>0</colOff>
-      <row>23</row>
-      <rowOff>0</rowOff>
-    </to>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="3" name="Chart 3"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1611,11 +1788,7 @@
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="1" t="n"/>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Independent holdout: quality and resource use</t>
-        </is>
-      </c>
+      <c r="B2" s="1" t="n"/>
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
       <c r="E2" s="1" t="n"/>
@@ -2165,22 +2338,22 @@
       <c r="U24" s="1" t="n"/>
       <c r="V24" s="1" t="n"/>
     </row>
-    <row r="25" ht="55" customHeight="1">
+    <row r="25" ht="42" customHeight="1">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Editable values and formulas: Data 2</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="8" t="n"/>
-      <c r="G25" s="8" t="n"/>
-      <c r="H25" s="8" t="n"/>
-      <c r="I25" s="8" t="n"/>
-      <c r="J25" s="1" t="n"/>
-      <c r="K25" s="1" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
+      <c r="J25" s="7" t="n"/>
+      <c r="K25" s="7" t="n"/>
       <c r="L25" s="1" t="n"/>
       <c r="M25" s="1" t="n"/>
       <c r="N25" s="1" t="n"/>
@@ -2193,18 +2366,18 @@
       <c r="U25" s="1" t="n"/>
       <c r="V25" s="1" t="n"/>
     </row>
-    <row r="26" ht="55" customHeight="1">
+    <row r="26" ht="42" customHeight="1">
       <c r="A26" s="1" t="n"/>
-      <c r="B26" s="9" t="n"/>
-      <c r="C26" s="13" t="n"/>
-      <c r="D26" s="13" t="n"/>
-      <c r="E26" s="9" t="n"/>
+      <c r="B26" s="12" t="n"/>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="12" t="n"/>
       <c r="F26" s="9" t="n"/>
       <c r="G26" s="9" t="n"/>
-      <c r="H26" s="14" t="n"/>
-      <c r="I26" s="14" t="n"/>
-      <c r="J26" s="15" t="n"/>
-      <c r="K26" s="1" t="n"/>
+      <c r="H26" s="13" t="n"/>
+      <c r="I26" s="13" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="9" t="n"/>
       <c r="L26" s="1" t="n"/>
       <c r="M26" s="1" t="n"/>
       <c r="N26" s="1" t="n"/>
@@ -2217,18 +2390,18 @@
       <c r="U26" s="1" t="n"/>
       <c r="V26" s="1" t="n"/>
     </row>
-    <row r="27" ht="55" customHeight="1">
+    <row r="27" ht="42" customHeight="1">
       <c r="A27" s="1" t="n"/>
-      <c r="B27" s="9" t="n"/>
-      <c r="C27" s="13" t="n"/>
-      <c r="D27" s="13" t="n"/>
-      <c r="E27" s="9" t="n"/>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
       <c r="F27" s="9" t="n"/>
       <c r="G27" s="9" t="n"/>
-      <c r="H27" s="14" t="n"/>
-      <c r="I27" s="14" t="n"/>
-      <c r="J27" s="15" t="n"/>
-      <c r="K27" s="1" t="n"/>
+      <c r="H27" s="13" t="n"/>
+      <c r="I27" s="13" t="n"/>
+      <c r="J27" s="9" t="n"/>
+      <c r="K27" s="9" t="n"/>
       <c r="L27" s="1" t="n"/>
       <c r="M27" s="1" t="n"/>
       <c r="N27" s="1" t="n"/>
@@ -2241,18 +2414,18 @@
       <c r="U27" s="1" t="n"/>
       <c r="V27" s="1" t="n"/>
     </row>
-    <row r="28" ht="55" customHeight="1">
+    <row r="28" ht="42" customHeight="1">
       <c r="A28" s="1" t="n"/>
-      <c r="B28" s="9" t="n"/>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
+      <c r="B28" s="12" t="n"/>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
       <c r="F28" s="9" t="n"/>
       <c r="G28" s="9" t="n"/>
-      <c r="H28" s="14" t="n"/>
-      <c r="I28" s="14" t="n"/>
-      <c r="J28" s="15" t="n"/>
-      <c r="K28" s="1" t="n"/>
+      <c r="H28" s="9" t="n"/>
+      <c r="I28" s="9" t="n"/>
+      <c r="J28" s="9" t="n"/>
+      <c r="K28" s="9" t="n"/>
       <c r="L28" s="1" t="n"/>
       <c r="M28" s="1" t="n"/>
       <c r="N28" s="1" t="n"/>
@@ -2393,7 +2566,7 @@
       <c r="E34" s="1" t="n"/>
       <c r="F34" s="1" t="n"/>
       <c r="G34" s="1" t="n"/>
-      <c r="H34" s="15" t="n"/>
+      <c r="H34" s="1" t="n"/>
       <c r="I34" s="1" t="n"/>
       <c r="J34" s="1" t="n"/>
       <c r="K34" s="1" t="n"/>
@@ -2740,11 +2913,7 @@
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="1" t="n"/>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Independent holdout: cohort comparison</t>
-        </is>
-      </c>
+      <c r="B2" s="1" t="n"/>
       <c r="C2" s="1" t="n"/>
       <c r="D2" s="1" t="n"/>
       <c r="E2" s="1" t="n"/>
@@ -3294,22 +3463,22 @@
       <c r="U24" s="1" t="n"/>
       <c r="V24" s="1" t="n"/>
     </row>
-    <row r="25" ht="55" customHeight="1">
+    <row r="25" ht="42" customHeight="1">
       <c r="A25" s="1" t="n"/>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Editable values and formulas: Data 3</t>
         </is>
       </c>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="8" t="n"/>
-      <c r="G25" s="8" t="n"/>
-      <c r="H25" s="8" t="n"/>
-      <c r="I25" s="8" t="n"/>
-      <c r="J25" s="1" t="n"/>
-      <c r="K25" s="1" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="7" t="n"/>
+      <c r="E25" s="7" t="n"/>
+      <c r="F25" s="7" t="n"/>
+      <c r="G25" s="7" t="n"/>
+      <c r="H25" s="7" t="n"/>
+      <c r="I25" s="7" t="n"/>
+      <c r="J25" s="7" t="n"/>
+      <c r="K25" s="7" t="n"/>
       <c r="L25" s="1" t="n"/>
       <c r="M25" s="1" t="n"/>
       <c r="N25" s="1" t="n"/>
@@ -3322,23 +3491,23 @@
       <c r="U25" s="1" t="n"/>
       <c r="V25" s="1" t="n"/>
     </row>
-    <row r="26" ht="55" customHeight="1">
+    <row r="26" ht="42" customHeight="1">
       <c r="A26" s="1" t="n"/>
       <c r="B26" s="9" t="n"/>
-      <c r="C26" s="9" t="n"/>
+      <c r="C26" s="14" t="n"/>
       <c r="D26" s="14" t="n"/>
-      <c r="E26" s="16" t="n"/>
-      <c r="F26" s="16" t="n"/>
-      <c r="G26" s="16" t="n"/>
+      <c r="E26" s="14" t="n"/>
+      <c r="F26" s="12" t="n"/>
+      <c r="G26" s="12" t="n"/>
       <c r="H26" s="14" t="n"/>
       <c r="I26" s="14" t="n"/>
-      <c r="J26" s="1" t="n"/>
-      <c r="K26" s="1" t="n"/>
+      <c r="J26" s="12" t="n"/>
+      <c r="K26" s="12" t="n"/>
       <c r="L26" s="1" t="n"/>
-      <c r="M26" s="1" t="n"/>
-      <c r="N26" s="1" t="n"/>
-      <c r="O26" s="1" t="n"/>
-      <c r="P26" s="1" t="n"/>
+      <c r="M26" s="15" t="n"/>
+      <c r="N26" s="15" t="n"/>
+      <c r="O26" s="15" t="n"/>
+      <c r="P26" s="15" t="n"/>
       <c r="Q26" s="1" t="n"/>
       <c r="R26" s="1" t="n"/>
       <c r="S26" s="1" t="n"/>
@@ -3346,23 +3515,23 @@
       <c r="U26" s="1" t="n"/>
       <c r="V26" s="1" t="n"/>
     </row>
-    <row r="27" ht="55" customHeight="1">
+    <row r="27" ht="42" customHeight="1">
       <c r="A27" s="1" t="n"/>
       <c r="B27" s="9" t="n"/>
-      <c r="C27" s="9" t="n"/>
+      <c r="C27" s="14" t="n"/>
       <c r="D27" s="14" t="n"/>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="16" t="n"/>
-      <c r="G27" s="16" t="n"/>
+      <c r="E27" s="14" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
       <c r="H27" s="14" t="n"/>
       <c r="I27" s="14" t="n"/>
-      <c r="J27" s="1" t="n"/>
-      <c r="K27" s="1" t="n"/>
+      <c r="J27" s="12" t="n"/>
+      <c r="K27" s="12" t="n"/>
       <c r="L27" s="1" t="n"/>
-      <c r="M27" s="1" t="n"/>
-      <c r="N27" s="1" t="n"/>
-      <c r="O27" s="1" t="n"/>
-      <c r="P27" s="1" t="n"/>
+      <c r="M27" s="15" t="n"/>
+      <c r="N27" s="15" t="n"/>
+      <c r="O27" s="15" t="n"/>
+      <c r="P27" s="15" t="n"/>
       <c r="Q27" s="1" t="n"/>
       <c r="R27" s="1" t="n"/>
       <c r="S27" s="1" t="n"/>
@@ -3370,23 +3539,23 @@
       <c r="U27" s="1" t="n"/>
       <c r="V27" s="1" t="n"/>
     </row>
-    <row r="28" ht="55" customHeight="1">
+    <row r="28" ht="42" customHeight="1">
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="9" t="n"/>
-      <c r="C28" s="9" t="n"/>
+      <c r="C28" s="14" t="n"/>
       <c r="D28" s="14" t="n"/>
-      <c r="E28" s="16" t="n"/>
-      <c r="F28" s="16" t="n"/>
-      <c r="G28" s="16" t="n"/>
+      <c r="E28" s="14" t="n"/>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="12" t="n"/>
       <c r="H28" s="14" t="n"/>
       <c r="I28" s="14" t="n"/>
-      <c r="J28" s="1" t="n"/>
-      <c r="K28" s="1" t="n"/>
+      <c r="J28" s="12" t="n"/>
+      <c r="K28" s="12" t="n"/>
       <c r="L28" s="1" t="n"/>
-      <c r="M28" s="1" t="n"/>
-      <c r="N28" s="1" t="n"/>
-      <c r="O28" s="1" t="n"/>
-      <c r="P28" s="1" t="n"/>
+      <c r="M28" s="15" t="n"/>
+      <c r="N28" s="15" t="n"/>
+      <c r="O28" s="15" t="n"/>
+      <c r="P28" s="15" t="n"/>
       <c r="Q28" s="1" t="n"/>
       <c r="R28" s="1" t="n"/>
       <c r="S28" s="1" t="n"/>
@@ -3816,7 +3985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B25:J38"/>
+  <dimension ref="B1:P14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="2" max="2"/>
@@ -3827,178 +3996,165 @@
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="25" ht="32" customHeight="1">
-      <c r="B25" s="17" t="inlineStr">
-        <is>
-          <t>Method</t>
-        </is>
-      </c>
-      <c r="C25" s="17" t="inlineStr">
-        <is>
-          <t>JEV tokens (millions)</t>
-        </is>
-      </c>
-      <c r="D25" s="17" t="inlineStr">
-        <is>
-          <t>L2 tokens (millions)</t>
-        </is>
-      </c>
-      <c r="G25" s="17" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Metric</t>
         </is>
       </c>
-      <c r="H25" s="17" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Point estimate</t>
         </is>
       </c>
-      <c r="I25" s="17" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>95% lower</t>
         </is>
       </c>
-      <c r="J25" s="18" t="inlineStr">
+      <c r="E1" s="16" t="inlineStr">
         <is>
           <t>95% upper</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="B26" s="18" t="inlineStr">
+      <c r="G1" s="16" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="H1" s="16" t="inlineStr">
+        <is>
+          <t>JEV</t>
+        </is>
+      </c>
+      <c r="I1" s="16" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="B2" s="17" t="inlineStr">
+        <is>
+          <t>Agreement</t>
+        </is>
+      </c>
+      <c r="C2" s="17" t="n">
+        <v>0.9774509803921568</v>
+      </c>
+      <c r="D2" s="17" t="n">
+        <v>0.9683116614151097</v>
+      </c>
+      <c r="E2" s="17" t="n">
+        <v>0.9867211440245148</v>
+      </c>
+      <c r="G2" s="18" t="inlineStr">
         <is>
           <t>Full L2</t>
         </is>
       </c>
-      <c r="C26" s="19" t="n">
+      <c r="H2" s="19" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="19" t="n">
+      <c r="I2" s="19" t="n">
         <v>2.750418</v>
       </c>
-      <c r="G26" s="18" t="inlineStr">
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="B3" s="17" t="inlineStr">
         <is>
-          <t>Agreement</t>
+          <t>Balanced agreement</t>
         </is>
       </c>
-      <c r="H26" s="20" t="n">
-        <v>0.9774509803921568</v>
-      </c>
-      <c r="I26" s="20" t="n">
-        <v>0.9683116614151097</v>
-      </c>
-      <c r="J26" s="20" t="n">
-        <v>0.9867211440245148</v>
-      </c>
-    </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="B27" s="18" t="inlineStr">
+      <c r="C3" s="17" t="n">
+        <v>0.9647567120853064</v>
+      </c>
+      <c r="D3" s="17" t="n">
+        <v>0.9348824046090382</v>
+      </c>
+      <c r="E3" s="17" t="n">
+        <v>0.9824114586278184</v>
+      </c>
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>Hybrid</t>
         </is>
       </c>
-      <c r="C27" s="19" t="n">
+      <c r="H3" s="19" t="n">
         <v>0.147061</v>
       </c>
-      <c r="D27" s="19" t="n">
+      <c r="I3" s="19" t="n">
         <v>0.7231919999999999</v>
       </c>
-      <c r="G27" s="18" t="inlineStr">
-        <is>
-          <t>Balanced agreement</t>
-        </is>
-      </c>
-      <c r="H27" s="20" t="n">
-        <v>0.9647567120853064</v>
-      </c>
-      <c r="I27" s="20" t="n">
-        <v>0.9348824046090382</v>
-      </c>
-      <c r="J27" s="20" t="n">
-        <v>0.9824114586278184</v>
-      </c>
-    </row>
-    <row r="28" ht="32" customHeight="1">
-      <c r="G28" s="18" t="inlineStr">
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="B4" s="17" t="inlineStr">
         <is>
           <t>Macro-F1</t>
         </is>
       </c>
-      <c r="H28" s="20" t="n">
+      <c r="C4" s="17" t="n">
         <v>0.9669720409742489</v>
       </c>
-      <c r="I28" s="20" t="n">
+      <c r="D4" s="17" t="n">
         <v>0.9389991288953802</v>
       </c>
-      <c r="J28" s="20" t="n">
+      <c r="E4" s="17" t="n">
         <v>0.9827630822315834</v>
       </c>
     </row>
-    <row r="29" ht="32" customHeight="1"/>
-    <row r="30" ht="32" customHeight="1"/>
-    <row r="31" ht="32" customHeight="1">
-      <c r="G31" s="18" t="inlineStr">
-        <is>
-          <t>Resource component</t>
-        </is>
-      </c>
-      <c r="H31" s="18" t="inlineStr">
-        <is>
-          <t>Tokens</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="32" customHeight="1">
-      <c r="G32" s="18" t="inlineStr">
-        <is>
-          <t>JEV</t>
-        </is>
-      </c>
-      <c r="H32" s="18" t="n">
-        <v>147061</v>
-      </c>
-    </row>
-    <row r="33" ht="32" customHeight="1">
-      <c r="G33" s="18" t="inlineStr">
-        <is>
-          <t>Selected L2</t>
-        </is>
-      </c>
-      <c r="H33" s="18" t="n">
-        <v>723192</v>
-      </c>
-    </row>
-    <row r="34" ht="32" customHeight="1">
-      <c r="G34" s="18" t="inlineStr">
-        <is>
-          <t>Token saving</t>
-        </is>
-      </c>
-      <c r="H34" s="20">
-        <f>1-(C27+D27)/D26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="35" ht="32" customHeight="1"/>
-    <row r="36" ht="32" customHeight="1"/>
-    <row r="37" ht="32" customHeight="1">
-      <c r="B37" s="18" t="inlineStr">
+    <row r="5" ht="32" customHeight="1"/>
+    <row r="6" ht="32" customHeight="1"/>
+    <row r="7" ht="32" customHeight="1"/>
+    <row r="8" ht="32" customHeight="1"/>
+    <row r="9" ht="32" customHeight="1"/>
+    <row r="10" ht="32" customHeight="1"/>
+    <row r="11" ht="32" customHeight="1"/>
+    <row r="12" ht="32" customHeight="1"/>
+    <row r="13" ht="32" customHeight="1">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>Source: independent holdout, 1,020 records from 100 household clusters.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="32" customHeight="1">
-      <c r="B38" s="18" t="inlineStr">
+    <row r="14" ht="32" customHeight="1">
+      <c r="B14" s="18" t="inlineStr">
         <is>
-          <t>Full-reference agreement measures the shared semantic contract; it is not observed-choice accuracy.</t>
+          <t>Filled bars are point estimates; hatched bars are 95% lower confidence bounds.</t>
         </is>
       </c>
     </row>
+    <row r="15" ht="32" customHeight="1"/>
+    <row r="25" ht="32" customHeight="1"/>
+    <row r="26" ht="32" customHeight="1"/>
+    <row r="27" ht="32" customHeight="1"/>
+    <row r="28" ht="32" customHeight="1"/>
+    <row r="29" ht="32" customHeight="1"/>
+    <row r="30" ht="32" customHeight="1"/>
+    <row r="31" ht="32" customHeight="1"/>
+    <row r="32" ht="32" customHeight="1"/>
+    <row r="33" ht="32" customHeight="1"/>
+    <row r="34" ht="32" customHeight="1"/>
+    <row r="35" ht="32" customHeight="1"/>
+    <row r="36" ht="32" customHeight="1"/>
+    <row r="37" ht="32" customHeight="1"/>
+    <row r="38" ht="32" customHeight="1"/>
     <row r="39" ht="32" customHeight="1"/>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B13:P13"/>
+    <mergeCell ref="B14:P14"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4009,7 +4165,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B25:I33"/>
+  <dimension ref="B1:P9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="2" max="2"/>
@@ -4020,157 +4176,248 @@
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
     <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="25" ht="32" customHeight="1">
-      <c r="B25" s="17" t="inlineStr">
+    <row r="1" ht="32" customHeight="1">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>Cohort</t>
         </is>
       </c>
-      <c r="C25" s="17" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>Records</t>
         </is>
       </c>
-      <c r="D25" s="17" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
+        <is>
+          <t>JEV calls</t>
+        </is>
+      </c>
+      <c r="E1" s="16" t="inlineStr">
+        <is>
+          <t>L2 calls</t>
+        </is>
+      </c>
+      <c r="F1" s="16" t="inlineStr">
+        <is>
+          <t>JEV</t>
+        </is>
+      </c>
+      <c r="G1" s="16" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="H1" s="16" t="inlineStr">
+        <is>
+          <t>Hybrid tokens</t>
+        </is>
+      </c>
+      <c r="I1" s="16" t="inlineStr">
+        <is>
+          <t>Full-L2 tokens</t>
+        </is>
+      </c>
+      <c r="J1" s="16" t="inlineStr">
+        <is>
+          <t>Token use ratio</t>
+        </is>
+      </c>
+      <c r="K1" s="16" t="inlineStr">
         <is>
           <t>Agreement</t>
         </is>
       </c>
-      <c r="E25" s="17" t="inlineStr">
+      <c r="M1" s="18" t="inlineStr">
         <is>
-          <t>Hybrid tokens</t>
+          <t>Token use ratio</t>
         </is>
       </c>
-      <c r="F25" s="17" t="inlineStr">
-        <is>
-          <t>Full-L2 tokens</t>
-        </is>
-      </c>
-      <c r="G25" s="17" t="inlineStr">
-        <is>
-          <t>L2 calls</t>
-        </is>
-      </c>
-      <c r="H25" s="17" t="inlineStr">
-        <is>
-          <t>Token saving</t>
-        </is>
-      </c>
-      <c r="I25" s="17" t="inlineStr">
-        <is>
-          <t>L2 rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="B26" s="18" t="inlineStr">
+      <c r="N1" s="18" t="inlineStr">
         <is>
           <t>Natural</t>
         </is>
       </c>
-      <c r="C26" s="18" t="n">
-        <v>400</v>
-      </c>
-      <c r="D26" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="21" t="n">
-        <v>118618</v>
-      </c>
-      <c r="F26" s="21" t="n">
-        <v>1060615</v>
-      </c>
-      <c r="G26" s="21" t="n">
-        <v>19</v>
-      </c>
-      <c r="H26" s="20">
-        <f>1-E26/F26</f>
-        <v/>
-      </c>
-      <c r="I26" s="20">
-        <f>G26/C26</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="B27" s="18" t="inlineStr">
+      <c r="O1" s="18" t="inlineStr">
         <is>
           <t>Stress</t>
         </is>
       </c>
-      <c r="C27" s="18" t="n">
-        <v>420</v>
-      </c>
-      <c r="D27" s="20" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="21" t="n">
-        <v>171724</v>
-      </c>
-      <c r="F27" s="21" t="n">
-        <v>1110033</v>
-      </c>
-      <c r="G27" s="21" t="n">
-        <v>34</v>
-      </c>
-      <c r="H27" s="20">
-        <f>1-E27/F27</f>
-        <v/>
-      </c>
-      <c r="I27" s="20">
-        <f>G27/C27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="32" customHeight="1">
-      <c r="B28" s="18" t="inlineStr">
+      <c r="P1" s="18" t="inlineStr">
         <is>
           <t>Policy OOD</t>
         </is>
       </c>
-      <c r="C28" s="18" t="n">
+    </row>
+    <row r="2" ht="32" customHeight="1">
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Natural</t>
+        </is>
+      </c>
+      <c r="C2" s="20" t="n">
+        <v>400</v>
+      </c>
+      <c r="D2" s="20" t="n">
+        <v>71</v>
+      </c>
+      <c r="E2" s="20" t="n">
+        <v>19</v>
+      </c>
+      <c r="F2" s="17">
+        <f>D2/C2</f>
+        <v/>
+      </c>
+      <c r="G2" s="17">
+        <f>E2/C2</f>
+        <v/>
+      </c>
+      <c r="H2" s="20" t="n">
+        <v>118618</v>
+      </c>
+      <c r="I2" s="20" t="n">
+        <v>1060615</v>
+      </c>
+      <c r="J2" s="17">
+        <f>H2/I2</f>
+        <v/>
+      </c>
+      <c r="K2" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" s="17" t="n">
+        <v>0.11183888592939</v>
+      </c>
+      <c r="N2" s="17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="B3" s="18" t="inlineStr">
+        <is>
+          <t>Stress</t>
+        </is>
+      </c>
+      <c r="C3" s="20" t="n">
+        <v>420</v>
+      </c>
+      <c r="D3" s="20" t="n">
+        <v>89</v>
+      </c>
+      <c r="E3" s="20" t="n">
+        <v>34</v>
+      </c>
+      <c r="F3" s="17">
+        <f>D3/C3</f>
+        <v/>
+      </c>
+      <c r="G3" s="17">
+        <f>E3/C3</f>
+        <v/>
+      </c>
+      <c r="H3" s="20" t="n">
+        <v>171724</v>
+      </c>
+      <c r="I3" s="20" t="n">
+        <v>1110033</v>
+      </c>
+      <c r="J3" s="17">
+        <f>H3/I3</f>
+        <v/>
+      </c>
+      <c r="K3" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" s="17" t="n">
+        <v>0.1547017070663665</v>
+      </c>
+      <c r="O3" s="17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="B4" s="18" t="inlineStr">
+        <is>
+          <t>Policy OOD</t>
+        </is>
+      </c>
+      <c r="C4" s="20" t="n">
         <v>200</v>
       </c>
-      <c r="D28" s="20" t="n">
+      <c r="D4" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="20" t="n">
+        <v>200</v>
+      </c>
+      <c r="F4" s="17">
+        <f>D4/C4</f>
+        <v/>
+      </c>
+      <c r="G4" s="17">
+        <f>E4/C4</f>
+        <v/>
+      </c>
+      <c r="H4" s="20" t="n">
+        <v>579911</v>
+      </c>
+      <c r="I4" s="20" t="n">
+        <v>579770</v>
+      </c>
+      <c r="J4" s="17">
+        <f>H4/I4</f>
+        <v/>
+      </c>
+      <c r="K4" s="17" t="n">
         <v>0.885</v>
       </c>
-      <c r="E28" s="21" t="n">
-        <v>579911</v>
-      </c>
-      <c r="F28" s="21" t="n">
-        <v>579770</v>
-      </c>
-      <c r="G28" s="21" t="n">
-        <v>200</v>
-      </c>
-      <c r="H28" s="20">
-        <f>1-E28/F28</f>
-        <v/>
-      </c>
-      <c r="I28" s="20">
-        <f>G28/C28</f>
-        <v/>
-      </c>
-    </row>
+      <c r="M4" s="17" t="n">
+        <v>1.000243199889611</v>
+      </c>
+      <c r="P4" s="17" t="n">
+        <v>0.885</v>
+      </c>
+    </row>
+    <row r="5" ht="32" customHeight="1"/>
+    <row r="6" ht="32" customHeight="1"/>
+    <row r="7" ht="32" customHeight="1"/>
+    <row r="8" ht="32" customHeight="1">
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Source: frozen independent holdout metrics; cohorts share household clusters.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="32" customHeight="1">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>Policy OOD uses 100.02% of full-L2 tokens because the two calls were executed independently.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1"/>
+    <row r="11" ht="32" customHeight="1"/>
+    <row r="12" ht="32" customHeight="1"/>
+    <row r="13" ht="32" customHeight="1"/>
+    <row r="14" ht="32" customHeight="1"/>
+    <row r="15" ht="32" customHeight="1"/>
+    <row r="25" ht="32" customHeight="1"/>
+    <row r="26" ht="32" customHeight="1"/>
+    <row r="27" ht="32" customHeight="1"/>
+    <row r="28" ht="32" customHeight="1"/>
     <row r="29" ht="32" customHeight="1"/>
     <row r="30" ht="32" customHeight="1"/>
     <row r="31" ht="32" customHeight="1"/>
-    <row r="32" ht="32" customHeight="1">
-      <c r="B32" s="18" t="inlineStr">
-        <is>
-          <t>Source: frozen independent holdout metrics; cohorts share household clusters.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="32" customHeight="1">
-      <c r="B33" s="18" t="inlineStr">
-        <is>
-          <t>Policy OOD token saving is -0.0243%; its rounded plotted value is -0.02%.</t>
-        </is>
-      </c>
-    </row>
+    <row r="32" ht="32" customHeight="1"/>
+    <row r="33" ht="32" customHeight="1"/>
     <row r="34" ht="32" customHeight="1"/>
     <row r="35" ht="32" customHeight="1"/>
     <row r="36" ht="32" customHeight="1"/>
@@ -4178,6 +4425,10 @@
     <row r="38" ht="32" customHeight="1"/>
     <row r="39" ht="32" customHeight="1"/>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B9:P9"/>
+    <mergeCell ref="B8:P8"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>